<commit_message>
change oppositionDate short ffe8e6cc1b312364f87b4ae42cbf7671db083d75
</commit_message>
<xml_diff>
--- a/nr-update-smart-card/ig/StructureDefinition-as-ext-smartcard.xlsx
+++ b/nr-update-smart-card/ig/StructureDefinition-as-ext-smartcard.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-18T12:44:27+00:00</t>
+    <t>2025-03-18T12:54:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -524,7 +524,7 @@
     <t>oppositionDate</t>
   </si>
   <si>
-    <t>dateOpposition : Date de mise en opposition de la carte.</t>
+    <t>dateOpposition : Date d'opposition de la carte.</t>
   </si>
   <si>
     <t>Extension.extension:oppositionDate.id</t>

</xml_diff>